<commit_message>
Add reconnect triggers/proactive reconnect, random-chat tab, human-verify auto-pass, quiz answer fixes (v2.1)
</commit_message>
<xml_diff>
--- a/玩家资料模板.xlsx
+++ b/玩家资料模板.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="27.7265625" customWidth="1" min="1" max="1"/>
@@ -540,27 +540,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>说话简短随性，爱用英文缩写，关心老玩家何时入服。</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>沉默寡言，爱用符号和化学式打哑谜的抽象谜语人。</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>爱跟人机验证较劲，认真答题，也爱发指令凑热闹。</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>话少爱刷单字母，偶尔认真问插件，像个闷声发财的老玩家。</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>服内富豪，热衷答题，偶尔冒问号，爱刷选项。</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>发言简短零碎，爱刷666和游戏梗，关注余额、缓存与答题的随性玩家。</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>寡言简语，爱用缩写，关注银行余额和数据缓存，偶尔喊666。</t>
         </is>
       </c>
     </row>
@@ -1073,27 +1073,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>友善健谈，熟悉服务器插件与经济，还能秒算轨道周期，随叫随到。</t>
+          <t>思维跳脱，爱发无厘头碎片词，常冒出编程、诗词和历史梗。</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>暴躁护短，脏话连篇，谁杀自己人或机器人就怒火冲天。</t>
+          <t>思维跳脱爱玩文字实验，常简短附和，话题杂糅随性。</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>发言极简跳脱，爱丢零散词和数字，显得神秘随性。</t>
+          <t>话少跳跃，热衷古风城建，常念叨坐标材料与规划，像沉浸式搞建设。</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>爱玩角色扮演与耕种，思维跳跃，常冒出月光曲、巨鹿、语义饱和等文艺词。</t>
+          <t>发言零碎抽象，常蹦数字和术语，像个沉迷调试的技术型玩家。</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>兴趣跳跃广泛，爱聊历史法律角色扮演，也喜欢种田和月光曲。</t>
+          <t>发言碎片化又跳脱，常答“对”，像爱蹦词和数字的谜语型玩家。</t>
         </is>
       </c>
     </row>
@@ -1348,6 +1348,18 @@
       <c r="J28" t="inlineStr">
         <is>
           <t>爱用文言文和文学史玩梗，自嘲作文差，常吐槽游戏税与房贷。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>HumanVerify</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>沉迷反复进出服务器并刷目标方块，像执着测试型的玩家。</t>
         </is>
       </c>
     </row>

</xml_diff>